<commit_message>
Update template file and add cache files
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Oguz\.qoder\n8n\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45DD7C0B-D0D0-4F28-9E65-59495CBE79F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D822A1-CAB0-4700-8D20-C479A6CCBDB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KACC" sheetId="4" r:id="rId1"/>
@@ -119,8 +119,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -453,28 +456,29 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E725000-1D6A-4DDD-B5B8-7764ADDD504D}">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K4055"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="8.88671875" style="1"/>
+    <col min="5" max="5" width="40.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="69.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F1" t="s">
@@ -496,8 +500,740 @@
         <v>9</v>
       </c>
     </row>
+    <row r="3342" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3342"/>
+      <c r="B3342"/>
+      <c r="C3342"/>
+      <c r="D3342"/>
+      <c r="E3342"/>
+    </row>
+    <row r="3343" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3343"/>
+      <c r="B3343"/>
+      <c r="C3343"/>
+      <c r="D3343"/>
+      <c r="E3343"/>
+    </row>
+    <row r="3344" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3344"/>
+      <c r="B3344"/>
+      <c r="C3344"/>
+      <c r="D3344"/>
+      <c r="E3344"/>
+    </row>
+    <row r="3345" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3346" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3347" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3348" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3349" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3350" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3351" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3352" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3353" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3354" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3355" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3356" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3357" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3358" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3359" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3360" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3361" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3362" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3363" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3364" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3365" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3366" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3367" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3368" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3369" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3370" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3371" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3372" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3373" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3374" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3375" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3376" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3377" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3378" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3379" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3380" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3381" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3382" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3383" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3384" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3385" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3386" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3387" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3388" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3389" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3390" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3391" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3392" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3393" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3394" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3395" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3396" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3397" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3398" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3399" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3400" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3401" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3402" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3403" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3404" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3405" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3406" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3407" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3408" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3409" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3410" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3411" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3412" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3413" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3414" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3415" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3416" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3417" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3418" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3419" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3420" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3421" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3422" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3423" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3424" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3425" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3426" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3427" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3428" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3429" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3430" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3431" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3432" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3433" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3434" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3435" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3436" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3437" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3438" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3439" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3440" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3441" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3442" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3443" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3444" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3445" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3446" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3447" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3448" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3449" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3450" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3451" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3452" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3453" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3454" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3455" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3456" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3457" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3458" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3459" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3460" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3461" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3462" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3463" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3464" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3465" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3466" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3467" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3468" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3469" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3470" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3471" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3472" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3473" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3474" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3475" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3476" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3477" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3478" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3479" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3480" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3481" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3482" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3483" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3484" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3485" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3486" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3487" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3488" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3489" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3490" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3491" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3492" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3493" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3494" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3495" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3496" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3497" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3498" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3499" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3500" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3501" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3502" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3503" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3504" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3505" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3506" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3507" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3508" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3509" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3510" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3511" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3512" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3513" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3514" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3515" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3516" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3517" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3518" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3519" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3520" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3521" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3522" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3523" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3524" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3525" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3526" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3527" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3528" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3529" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3530" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3531" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3532" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3533" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3534" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3535" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3536" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3537" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3538" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3539" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3540" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3541" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3542" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3543" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3544" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3545" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3546" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3547" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3548" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3549" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3550" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3551" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3552" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3553" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3554" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3555" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3556" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3557" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3558" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3559" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3560" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3561" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3562" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3563" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3564" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3565" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3566" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3567" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3568" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3569" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3570" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3571" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3572" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3573" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3574" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3575" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3576" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3577" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3578" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3579" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3580" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3581" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3582" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3583" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3584" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3585" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3586" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3587" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3588" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3589" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3590" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3591" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3592" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3593" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3594" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3595" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3596" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3597" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3598" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3599" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3600" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3601" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3602" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3603" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3604" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3605" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3606" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3607" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3608" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3609" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3610" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3611" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3612" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3613" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3614" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3615" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3616" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3617" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3618" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3619" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3620" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3621" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3622" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3623" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3624" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3625" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3626" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3627" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3628" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3629" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3630" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3631" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3632" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3633" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3634" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3635" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3636" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3637" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3638" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3639" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3640" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3641" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3642" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3643" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3644" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3645" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3646" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3647" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3648" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3649" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3650" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3651" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3652" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3653" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3654" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3655" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3656" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3657" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3658" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3659" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3660" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3661" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3662" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3663" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3664" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3665" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3666" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3667" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3668" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3669" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3670" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3671" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3672" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3673" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3674" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3675" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3676" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3677" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3678" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3679" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3680" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3681" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3682" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3683" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3684" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3685" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3686" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3687" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3688" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3689" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3690" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3691" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3692" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3693" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3694" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3695" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3696" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3697" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3698" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3699" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3700" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3701" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3702" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3703" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3704" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3705" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3706" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3707" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3708" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3709" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3710" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3711" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3712" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3713" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3714" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3715" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3716" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3717" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3718" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3719" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3720" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3721" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3722" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3723" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3724" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3725" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3726" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3727" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3728" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3729" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3730" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3731" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3732" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3733" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3734" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3735" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3736" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3737" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3738" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3739" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3740" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3741" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3742" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3743" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3744" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3745" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3746" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3747" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3748" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3749" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3750" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3751" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3752" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3753" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3754" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3755" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3756" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3757" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3758" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3759" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3760" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3761" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3762" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3763" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3764" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3765" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3766" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3767" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3768" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3769" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3770" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3771" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3772" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3773" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3774" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3775" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3776" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3777" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3778" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3779" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3780" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3781" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3782" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3783" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3784" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3785" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3786" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3787" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3788" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3789" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3790" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3791" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3792" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3793" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3794" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3795" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3796" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3797" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3798" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3799" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3800" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3801" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3802" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3803" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3804" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3805" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3806" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3807" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3808" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3809" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3810" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3811" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3812" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3813" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3814" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3815" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3816" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3817" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3818" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3819" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3820" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3821" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3822" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3823" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3824" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3825" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3826" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3827" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3828" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3829" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3830" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3831" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3832" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3833" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3834" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3835" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3836" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3837" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3838" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3839" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3840" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3841" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3842" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3843" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3844" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3845" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3846" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3847" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3848" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3849" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3850" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3851" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3852" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3853" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3854" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3855" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3856" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3857" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3858" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3859" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3860" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3861" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3862" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3863" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3864" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3865" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3866" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3867" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3868" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3869" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3870" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3871" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3872" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3873" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3874" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3875" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3876" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3877" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3878" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3879" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3880" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3881" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3882" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3883" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3884" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3885" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3886" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3887" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3888" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3889" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3890" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3891" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3892" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3893" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3894" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3895" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3896" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3897" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3898" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3899" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3900" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3901" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3902" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3903" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3904" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3905" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3906" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3907" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3908" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3909" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3910" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3911" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3912" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3913" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3914" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3915" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3916" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3917" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3918" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3919" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3920" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3921" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3922" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3923" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3924" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3925" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3926" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3927" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3928" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3929" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3930" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3931" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3932" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3933" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3934" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3935" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3936" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3937" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3938" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3939" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3940" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3941" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3942" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3943" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3944" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3945" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3946" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3947" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3948" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3949" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3950" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3951" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3952" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3953" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3954" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3955" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3956" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3957" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3958" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3959" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3960" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3961" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3962" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3963" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3964" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3965" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3966" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3967" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3968" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3969" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3970" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3971" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3972" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3973" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3974" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3975" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3976" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3977" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3978" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3979" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3980" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3981" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3982" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3983" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3984" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3985" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3986" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3987" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3988" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3989" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3990" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3991" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3992" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3993" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3994" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3995" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3996" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3997" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3998" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="3999" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4000" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4001" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4002" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4003" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4004" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4005" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4006" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4007" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4008" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4009" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4010" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4011" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4012" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4013" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4014" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4015" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4016" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4017" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4018" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4019" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4020" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4021" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4022" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4023" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4024" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4025" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4026" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4027" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4028" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4029" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4030" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4031" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4032" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4033" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4034" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4035" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4036" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4037" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4038" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4039" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4040" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4041" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4042" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4043" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4044" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4045" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4046" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4047" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4048" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4049" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4050" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4051" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4052" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4053" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4054" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="4055" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A1:K1" xr:uid="{8E725000-1D6A-4DDD-B5B8-7764ADDD504D}"/>
+  <autoFilter ref="A1:K3341" xr:uid="{8E725000-1D6A-4DDD-B5B8-7764ADDD504D}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>